<commit_message>
updating things but taking a pause
</commit_message>
<xml_diff>
--- a/390-semester-planner.xlsx
+++ b/390-semester-planner.xlsx
@@ -109,7 +109,7 @@
     <numFmt numFmtId="168" formatCode="@"/>
     <numFmt numFmtId="169" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -160,12 +160,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Open Sans"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -289,7 +283,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -404,10 +398,6 @@
     </xf>
     <xf numFmtId="168" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1020,9 +1010,7 @@
       </c>
       <c r="G14" s="21"/>
       <c r="J14" s="22"/>
-      <c r="K14" s="22" t="s">
-        <v>17</v>
-      </c>
+      <c r="K14" s="22"/>
       <c r="L14" s="15"/>
       <c r="N14" s="1" t="n">
         <v>9</v>
@@ -1068,8 +1056,8 @@
       <c r="J16" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="K16" s="22" t="n">
-        <v>4</v>
+      <c r="K16" s="22" t="s">
+        <v>17</v>
       </c>
       <c r="L16" s="15"/>
       <c r="N16" s="1" t="n">
@@ -1110,7 +1098,7 @@
         <f aca="false">IF(D17="",D16+IF(OR(WEEKDAY(D16)=2,WEEKDAY(D16)=4),2,3),"")</f>
         <v>45905</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="25" t="s">
         <v>18</v>
       </c>
       <c r="F18" s="26"/>
@@ -1118,9 +1106,7 @@
       <c r="J18" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="K18" s="22" t="s">
-        <v>19</v>
-      </c>
+      <c r="K18" s="22"/>
       <c r="L18" s="15"/>
       <c r="N18" s="1" t="n">
         <v>13</v>
@@ -1134,7 +1120,7 @@
       <c r="B19" s="17"/>
       <c r="C19" s="22"/>
       <c r="D19" s="24"/>
-      <c r="E19" s="29"/>
+      <c r="E19" s="25"/>
       <c r="F19" s="26"/>
       <c r="G19" s="21"/>
       <c r="J19" s="22"/>
@@ -1168,9 +1154,7 @@
       <c r="J20" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="K20" s="22" t="s">
-        <v>20</v>
-      </c>
+      <c r="K20" s="22"/>
       <c r="L20" s="15"/>
       <c r="N20" s="1" t="n">
         <v>15</v>
@@ -1215,7 +1199,7 @@
         <v>7</v>
       </c>
       <c r="K22" s="22" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L22" s="15"/>
       <c r="N22" s="1" t="n">
@@ -1263,9 +1247,8 @@
         <f aca="false">J22+1</f>
         <v>8</v>
       </c>
-      <c r="K24" s="22" t="n">
-        <f aca="false">K22+1</f>
-        <v>8</v>
+      <c r="K24" s="22" t="s">
+        <v>19</v>
       </c>
       <c r="L24" s="15"/>
       <c r="N24" s="1" t="n">
@@ -1297,7 +1280,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
-      <c r="B26" s="30" t="n">
+      <c r="B26" s="29" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="17" t="n">
@@ -1315,9 +1298,8 @@
         <f aca="false">J24+1</f>
         <v>9</v>
       </c>
-      <c r="K26" s="22" t="n">
-        <f aca="false">K24+1</f>
-        <v>9</v>
+      <c r="K26" s="22" t="s">
+        <v>20</v>
       </c>
       <c r="L26" s="15"/>
       <c r="N26" s="1" t="n">
@@ -1330,7 +1312,7 @@
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2"/>
-      <c r="B27" s="30"/>
+      <c r="B27" s="29"/>
       <c r="C27" s="17"/>
       <c r="D27" s="18"/>
       <c r="E27" s="19"/>
@@ -1349,7 +1331,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
-      <c r="B28" s="30"/>
+      <c r="B28" s="29"/>
       <c r="C28" s="22" t="n">
         <f aca="false">C26+1</f>
         <v>10</v>
@@ -1365,10 +1347,7 @@
         <f aca="false">J26+1</f>
         <v>10</v>
       </c>
-      <c r="K28" s="22" t="n">
-        <f aca="false">K26+1</f>
-        <v>10</v>
-      </c>
+      <c r="K28" s="22"/>
       <c r="L28" s="15"/>
       <c r="N28" s="1" t="n">
         <v>23</v>
@@ -1380,7 +1359,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2"/>
-      <c r="B29" s="30"/>
+      <c r="B29" s="29"/>
       <c r="C29" s="22"/>
       <c r="D29" s="24"/>
       <c r="E29" s="25"/>
@@ -1399,26 +1378,23 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="31" t="n">
+      <c r="B30" s="29"/>
+      <c r="C30" s="30" t="n">
         <f aca="false">C28+1</f>
         <v>11</v>
       </c>
-      <c r="D30" s="32" t="n">
+      <c r="D30" s="31" t="n">
         <f aca="false">IF(D29="",D28+IF(OR(WEEKDAY(D28)=2,WEEKDAY(D28)=4),2,3),"")</f>
         <v>45919</v>
       </c>
       <c r="E30" s="25"/>
-      <c r="F30" s="33"/>
+      <c r="F30" s="32"/>
       <c r="G30" s="21"/>
       <c r="J30" s="22" t="n">
         <f aca="false">J28+1</f>
         <v>11</v>
       </c>
-      <c r="K30" s="22" t="n">
-        <f aca="false">K28+1</f>
-        <v>11</v>
-      </c>
+      <c r="K30" s="22"/>
       <c r="L30" s="15"/>
       <c r="N30" s="1" t="n">
         <v>25</v>
@@ -1429,11 +1405,11 @@
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
-      <c r="B31" s="30"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="32"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="30"/>
+      <c r="D31" s="31"/>
       <c r="E31" s="25"/>
-      <c r="F31" s="33"/>
+      <c r="F31" s="32"/>
       <c r="G31" s="21"/>
       <c r="J31" s="22"/>
       <c r="K31" s="22"/>
@@ -1447,7 +1423,7 @@
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2"/>
-      <c r="B32" s="30" t="n">
+      <c r="B32" s="29" t="n">
         <v>5</v>
       </c>
       <c r="C32" s="17" t="n">
@@ -1460,15 +1436,12 @@
       </c>
       <c r="E32" s="19"/>
       <c r="F32" s="20"/>
-      <c r="G32" s="34"/>
+      <c r="G32" s="33"/>
       <c r="J32" s="22" t="n">
         <f aca="false">J30+1</f>
         <v>12</v>
       </c>
-      <c r="K32" s="22" t="n">
-        <f aca="false">K30+1</f>
-        <v>12</v>
-      </c>
+      <c r="K32" s="22"/>
       <c r="L32" s="15"/>
       <c r="N32" s="1" t="n">
         <v>27</v>
@@ -1479,7 +1452,7 @@
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2"/>
-      <c r="B33" s="30"/>
+      <c r="B33" s="29"/>
       <c r="C33" s="17"/>
       <c r="D33" s="18"/>
       <c r="E33" s="19"/>
@@ -1497,7 +1470,7 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="30"/>
+      <c r="B34" s="29"/>
       <c r="C34" s="22" t="n">
         <f aca="false">C32+1</f>
         <v>13</v>
@@ -1508,15 +1481,12 @@
       </c>
       <c r="E34" s="25"/>
       <c r="F34" s="26"/>
-      <c r="G34" s="34"/>
+      <c r="G34" s="33"/>
       <c r="J34" s="22" t="n">
         <f aca="false">J32+1</f>
         <v>13</v>
       </c>
-      <c r="K34" s="22" t="n">
-        <f aca="false">K32+1</f>
-        <v>13</v>
-      </c>
+      <c r="K34" s="22"/>
       <c r="L34" s="15"/>
       <c r="N34" s="1" t="n">
         <v>29</v>
@@ -1528,7 +1498,7 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2"/>
-      <c r="B35" s="30"/>
+      <c r="B35" s="29"/>
       <c r="C35" s="22"/>
       <c r="D35" s="24"/>
       <c r="E35" s="25"/>
@@ -1547,26 +1517,23 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2"/>
-      <c r="B36" s="30"/>
-      <c r="C36" s="31" t="n">
+      <c r="B36" s="29"/>
+      <c r="C36" s="30" t="n">
         <f aca="false">C34+1</f>
         <v>14</v>
       </c>
-      <c r="D36" s="32" t="n">
+      <c r="D36" s="31" t="n">
         <f aca="false">IF(D35="",D34+IF(OR(WEEKDAY(D34)=2,WEEKDAY(D34)=4),2,3),"")</f>
         <v>45926</v>
       </c>
       <c r="E36" s="25"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="34"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="33"/>
       <c r="J36" s="22" t="n">
         <f aca="false">J34+1</f>
         <v>14</v>
       </c>
-      <c r="K36" s="22" t="n">
-        <f aca="false">K34+1</f>
-        <v>14</v>
-      </c>
+      <c r="K36" s="22"/>
       <c r="L36" s="15"/>
       <c r="N36" s="1" t="n">
         <v>31</v>
@@ -1577,12 +1544,12 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2"/>
-      <c r="B37" s="30"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="32"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="31"/>
       <c r="E37" s="25"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="34"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="33"/>
       <c r="J37" s="22"/>
       <c r="K37" s="22"/>
       <c r="L37" s="15"/>
@@ -1596,7 +1563,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2"/>
-      <c r="B38" s="30" t="n">
+      <c r="B38" s="29" t="n">
         <v>6</v>
       </c>
       <c r="C38" s="17" t="n">
@@ -1609,15 +1576,12 @@
       </c>
       <c r="E38" s="19"/>
       <c r="F38" s="20"/>
-      <c r="G38" s="34"/>
+      <c r="G38" s="33"/>
       <c r="J38" s="22" t="n">
         <f aca="false">J36+1</f>
         <v>15</v>
       </c>
-      <c r="K38" s="22" t="n">
-        <f aca="false">K36+1</f>
-        <v>15</v>
-      </c>
+      <c r="K38" s="22"/>
       <c r="L38" s="15"/>
       <c r="N38" s="1" t="n">
         <v>33</v>
@@ -1629,12 +1593,12 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2"/>
-      <c r="B39" s="30"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="17"/>
       <c r="D39" s="18"/>
       <c r="E39" s="19"/>
       <c r="F39" s="20"/>
-      <c r="G39" s="34"/>
+      <c r="G39" s="33"/>
       <c r="J39" s="22"/>
       <c r="K39" s="22"/>
       <c r="L39" s="15"/>
@@ -1648,7 +1612,7 @@
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
-      <c r="B40" s="30"/>
+      <c r="B40" s="29"/>
       <c r="C40" s="22" t="n">
         <f aca="false">C38+1</f>
         <v>16</v>
@@ -1659,15 +1623,12 @@
       </c>
       <c r="E40" s="25"/>
       <c r="F40" s="26"/>
-      <c r="G40" s="34"/>
+      <c r="G40" s="33"/>
       <c r="J40" s="22" t="n">
         <f aca="false">J38+1</f>
         <v>16</v>
       </c>
-      <c r="K40" s="22" t="n">
-        <f aca="false">K38+1</f>
-        <v>16</v>
-      </c>
+      <c r="K40" s="22"/>
       <c r="L40" s="15"/>
       <c r="N40" s="1" t="n">
         <v>35</v>
@@ -1678,12 +1639,12 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2"/>
-      <c r="B41" s="30"/>
+      <c r="B41" s="29"/>
       <c r="C41" s="22"/>
       <c r="D41" s="24"/>
       <c r="E41" s="25"/>
       <c r="F41" s="26"/>
-      <c r="G41" s="34"/>
+      <c r="G41" s="33"/>
       <c r="J41" s="22"/>
       <c r="K41" s="22"/>
       <c r="L41" s="15"/>
@@ -1697,26 +1658,23 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="31" t="n">
+      <c r="B42" s="29"/>
+      <c r="C42" s="30" t="n">
         <f aca="false">C40+1</f>
         <v>17</v>
       </c>
-      <c r="D42" s="32" t="n">
+      <c r="D42" s="31" t="n">
         <f aca="false">IF(D41="",D40+IF(OR(WEEKDAY(D40)=2,WEEKDAY(D40)=4),2,3),"")</f>
         <v>45933</v>
       </c>
       <c r="E42" s="25"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="34"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="33"/>
       <c r="J42" s="22" t="n">
         <f aca="false">J40+1</f>
         <v>17</v>
       </c>
-      <c r="K42" s="22" t="n">
-        <f aca="false">K40+1</f>
-        <v>17</v>
-      </c>
+      <c r="K42" s="22"/>
       <c r="L42" s="15"/>
       <c r="N42" s="1" t="n">
         <v>37</v>
@@ -1728,12 +1686,12 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="32"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="31"/>
       <c r="E43" s="25"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="34"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="33"/>
       <c r="J43" s="22"/>
       <c r="K43" s="22"/>
       <c r="L43" s="15"/>
@@ -1750,7 +1708,7 @@
         <f aca="false">DATE(D3,D4+2,1)</f>
         <v>45931</v>
       </c>
-      <c r="B44" s="30" t="n">
+      <c r="B44" s="29" t="n">
         <v>7</v>
       </c>
       <c r="C44" s="17" t="n">
@@ -1768,10 +1726,7 @@
         <f aca="false">J42+1</f>
         <v>18</v>
       </c>
-      <c r="K44" s="22" t="n">
-        <f aca="false">K42+1</f>
-        <v>18</v>
-      </c>
+      <c r="K44" s="22"/>
       <c r="L44" s="15"/>
       <c r="N44" s="1" t="n">
         <v>39</v>
@@ -1783,7 +1738,7 @@
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2"/>
-      <c r="B45" s="30"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="17"/>
       <c r="D45" s="18"/>
       <c r="E45" s="19"/>
@@ -1802,7 +1757,7 @@
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2"/>
-      <c r="B46" s="30"/>
+      <c r="B46" s="29"/>
       <c r="C46" s="22" t="n">
         <f aca="false">C44+1</f>
         <v>19</v>
@@ -1818,10 +1773,7 @@
         <f aca="false">J44+1</f>
         <v>19</v>
       </c>
-      <c r="K46" s="22" t="n">
-        <f aca="false">K44+1</f>
-        <v>19</v>
-      </c>
+      <c r="K46" s="22"/>
       <c r="L46" s="15"/>
       <c r="N46" s="1" t="n">
         <v>41</v>
@@ -1832,7 +1784,7 @@
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2"/>
-      <c r="B47" s="30"/>
+      <c r="B47" s="29"/>
       <c r="C47" s="22"/>
       <c r="D47" s="24"/>
       <c r="E47" s="25"/>
@@ -1851,26 +1803,23 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2"/>
-      <c r="B48" s="30"/>
-      <c r="C48" s="31" t="n">
+      <c r="B48" s="29"/>
+      <c r="C48" s="30" t="n">
         <f aca="false">C46+1</f>
         <v>20</v>
       </c>
-      <c r="D48" s="32" t="n">
+      <c r="D48" s="31" t="n">
         <f aca="false">IF(D47="",D46+IF(OR(WEEKDAY(D46)=2,WEEKDAY(D46)=4),2,3),"")</f>
         <v>45940</v>
       </c>
       <c r="E48" s="25"/>
-      <c r="F48" s="33"/>
+      <c r="F48" s="32"/>
       <c r="G48" s="21"/>
       <c r="J48" s="22" t="n">
         <f aca="false">J46+1</f>
         <v>20</v>
       </c>
-      <c r="K48" s="22" t="n">
-        <f aca="false">K46+1</f>
-        <v>20</v>
-      </c>
+      <c r="K48" s="22"/>
       <c r="L48" s="15"/>
       <c r="N48" s="1" t="n">
         <v>43</v>
@@ -1882,11 +1831,11 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2"/>
-      <c r="B49" s="30"/>
-      <c r="C49" s="31"/>
-      <c r="D49" s="32"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="31"/>
       <c r="E49" s="25"/>
-      <c r="F49" s="33"/>
+      <c r="F49" s="32"/>
       <c r="G49" s="21"/>
       <c r="J49" s="22"/>
       <c r="K49" s="22"/>
@@ -1959,9 +1908,7 @@
       <c r="J52" s="22" t="n">
         <v>21</v>
       </c>
-      <c r="K52" s="22" t="n">
-        <v>21</v>
-      </c>
+      <c r="K52" s="22"/>
       <c r="L52" s="15"/>
       <c r="N52" s="1" t="n">
         <v>47</v>
@@ -2001,10 +1948,7 @@
         <f aca="false">J52+1</f>
         <v>22</v>
       </c>
-      <c r="K54" s="22" t="n">
-        <f aca="false">K52+1</f>
-        <v>22</v>
-      </c>
+      <c r="K54" s="22"/>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2"/>
@@ -2019,7 +1963,7 @@
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2"/>
-      <c r="B56" s="30" t="n">
+      <c r="B56" s="29" t="n">
         <v>9</v>
       </c>
       <c r="C56" s="17" t="n">
@@ -2037,14 +1981,11 @@
         <f aca="false">J54+1</f>
         <v>23</v>
       </c>
-      <c r="K56" s="22" t="n">
-        <f aca="false">K54+1</f>
-        <v>23</v>
-      </c>
+      <c r="K56" s="22"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2"/>
-      <c r="B57" s="30"/>
+      <c r="B57" s="29"/>
       <c r="C57" s="17"/>
       <c r="D57" s="18"/>
       <c r="E57" s="19"/>
@@ -2055,7 +1996,7 @@
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2"/>
-      <c r="B58" s="30"/>
+      <c r="B58" s="29"/>
       <c r="C58" s="22" t="n">
         <f aca="false">C56+1</f>
         <v>24</v>
@@ -2071,14 +2012,11 @@
         <f aca="false">J56+1</f>
         <v>24</v>
       </c>
-      <c r="K58" s="22" t="n">
-        <f aca="false">K56+1</f>
-        <v>24</v>
-      </c>
+      <c r="K58" s="22"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2"/>
-      <c r="B59" s="30"/>
+      <c r="B59" s="29"/>
       <c r="C59" s="22"/>
       <c r="D59" s="24"/>
       <c r="E59" s="25"/>
@@ -2088,41 +2026,38 @@
       <c r="K59" s="22"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="30"/>
-      <c r="C60" s="31" t="n">
+      <c r="B60" s="29"/>
+      <c r="C60" s="30" t="n">
         <f aca="false">C58+1</f>
         <v>25</v>
       </c>
-      <c r="D60" s="32" t="n">
+      <c r="D60" s="31" t="n">
         <f aca="false">IF(D59="",D58+IF(OR(WEEKDAY(D58)=2,WEEKDAY(D58)=4),2,3),"")</f>
         <v>45954</v>
       </c>
       <c r="E60" s="25"/>
-      <c r="F60" s="33"/>
+      <c r="F60" s="32"/>
       <c r="G60" s="21"/>
       <c r="J60" s="22" t="n">
         <f aca="false">J58+1</f>
         <v>25</v>
       </c>
-      <c r="K60" s="22" t="n">
-        <f aca="false">K58+1</f>
-        <v>25</v>
-      </c>
+      <c r="K60" s="22"/>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2"/>
-      <c r="B61" s="30"/>
-      <c r="C61" s="31"/>
-      <c r="D61" s="32"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="30"/>
+      <c r="D61" s="31"/>
       <c r="E61" s="25"/>
-      <c r="F61" s="33"/>
+      <c r="F61" s="32"/>
       <c r="G61" s="21"/>
       <c r="J61" s="22"/>
       <c r="K61" s="22"/>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2"/>
-      <c r="B62" s="30" t="n">
+      <c r="B62" s="29" t="n">
         <v>10</v>
       </c>
       <c r="C62" s="17" t="n">
@@ -2140,14 +2075,11 @@
         <f aca="false">J60+1</f>
         <v>26</v>
       </c>
-      <c r="K62" s="22" t="n">
-        <f aca="false">K60+1</f>
-        <v>26</v>
-      </c>
+      <c r="K62" s="22"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2"/>
-      <c r="B63" s="30"/>
+      <c r="B63" s="29"/>
       <c r="C63" s="17"/>
       <c r="D63" s="18"/>
       <c r="E63" s="19"/>
@@ -2158,7 +2090,7 @@
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2"/>
-      <c r="B64" s="30"/>
+      <c r="B64" s="29"/>
       <c r="C64" s="22" t="n">
         <f aca="false">C62+1</f>
         <v>27</v>
@@ -2174,14 +2106,11 @@
         <f aca="false">J62+1</f>
         <v>27</v>
       </c>
-      <c r="K64" s="22" t="n">
-        <f aca="false">K62+1</f>
-        <v>27</v>
-      </c>
+      <c r="K64" s="22"/>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2"/>
-      <c r="B65" s="30"/>
+      <c r="B65" s="29"/>
       <c r="C65" s="22"/>
       <c r="D65" s="24"/>
       <c r="E65" s="25"/>
@@ -2192,41 +2121,38 @@
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2"/>
-      <c r="B66" s="30"/>
-      <c r="C66" s="31" t="n">
+      <c r="B66" s="29"/>
+      <c r="C66" s="30" t="n">
         <f aca="false">C64+1</f>
         <v>28</v>
       </c>
-      <c r="D66" s="32" t="n">
+      <c r="D66" s="31" t="n">
         <f aca="false">IF(D65="",D64+IF(OR(WEEKDAY(D64)=2,WEEKDAY(D64)=4),2,3),"")</f>
         <v>45961</v>
       </c>
       <c r="E66" s="25"/>
-      <c r="F66" s="33"/>
+      <c r="F66" s="32"/>
       <c r="G66" s="21"/>
       <c r="J66" s="22" t="n">
         <f aca="false">J64+1</f>
         <v>28</v>
       </c>
-      <c r="K66" s="22" t="n">
-        <f aca="false">K64+1</f>
-        <v>28</v>
-      </c>
+      <c r="K66" s="22"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2"/>
-      <c r="B67" s="30"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="32"/>
+      <c r="B67" s="29"/>
+      <c r="C67" s="30"/>
+      <c r="D67" s="31"/>
       <c r="E67" s="25"/>
-      <c r="F67" s="33"/>
+      <c r="F67" s="32"/>
       <c r="G67" s="21"/>
       <c r="J67" s="22"/>
       <c r="K67" s="22"/>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2"/>
-      <c r="B68" s="30" t="n">
+      <c r="B68" s="29" t="n">
         <v>11</v>
       </c>
       <c r="C68" s="17" t="n">
@@ -2244,14 +2170,11 @@
         <f aca="false">J66+1</f>
         <v>29</v>
       </c>
-      <c r="K68" s="22" t="n">
-        <f aca="false">K66+1</f>
-        <v>29</v>
-      </c>
+      <c r="K68" s="22"/>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2"/>
-      <c r="B69" s="30"/>
+      <c r="B69" s="29"/>
       <c r="C69" s="17"/>
       <c r="D69" s="18"/>
       <c r="E69" s="19"/>
@@ -2265,7 +2188,7 @@
         <f aca="false">DATE(D3,D4+3,1)</f>
         <v>45962</v>
       </c>
-      <c r="B70" s="30"/>
+      <c r="B70" s="29"/>
       <c r="C70" s="22" t="n">
         <f aca="false">C68+1</f>
         <v>30</v>
@@ -2281,14 +2204,11 @@
         <f aca="false">J68+1</f>
         <v>30</v>
       </c>
-      <c r="K70" s="22" t="n">
-        <f aca="false">K68+1</f>
-        <v>30</v>
-      </c>
+      <c r="K70" s="22"/>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2"/>
-      <c r="B71" s="30"/>
+      <c r="B71" s="29"/>
       <c r="C71" s="22"/>
       <c r="D71" s="24"/>
       <c r="E71" s="25"/>
@@ -2299,41 +2219,38 @@
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2"/>
-      <c r="B72" s="30"/>
-      <c r="C72" s="31" t="n">
+      <c r="B72" s="29"/>
+      <c r="C72" s="30" t="n">
         <f aca="false">C70+1</f>
         <v>31</v>
       </c>
-      <c r="D72" s="32" t="n">
+      <c r="D72" s="31" t="n">
         <f aca="false">IF(D71="",D70+IF(OR(WEEKDAY(D70)=2,WEEKDAY(D70)=4),2,3),"")</f>
         <v>45968</v>
       </c>
       <c r="E72" s="25"/>
-      <c r="F72" s="33"/>
+      <c r="F72" s="32"/>
       <c r="G72" s="21"/>
       <c r="J72" s="22" t="n">
         <f aca="false">J70+1</f>
         <v>31</v>
       </c>
-      <c r="K72" s="22" t="n">
-        <f aca="false">K70+1</f>
-        <v>31</v>
-      </c>
+      <c r="K72" s="22"/>
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2"/>
-      <c r="B73" s="30"/>
-      <c r="C73" s="31"/>
-      <c r="D73" s="32"/>
+      <c r="B73" s="29"/>
+      <c r="C73" s="30"/>
+      <c r="D73" s="31"/>
       <c r="E73" s="25"/>
-      <c r="F73" s="33"/>
+      <c r="F73" s="32"/>
       <c r="G73" s="21"/>
       <c r="J73" s="22"/>
       <c r="K73" s="22"/>
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2"/>
-      <c r="B74" s="30" t="n">
+      <c r="B74" s="29" t="n">
         <v>12</v>
       </c>
       <c r="C74" s="17" t="n">
@@ -2351,14 +2268,11 @@
         <f aca="false">J72+1</f>
         <v>32</v>
       </c>
-      <c r="K74" s="22" t="n">
-        <f aca="false">K72+1</f>
-        <v>32</v>
-      </c>
+      <c r="K74" s="22"/>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2"/>
-      <c r="B75" s="30"/>
+      <c r="B75" s="29"/>
       <c r="C75" s="17"/>
       <c r="D75" s="18"/>
       <c r="E75" s="19"/>
@@ -2369,7 +2283,7 @@
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2"/>
-      <c r="B76" s="30"/>
+      <c r="B76" s="29"/>
       <c r="C76" s="22" t="n">
         <f aca="false">C74+1</f>
         <v>33</v>
@@ -2385,14 +2299,11 @@
         <f aca="false">J74+1</f>
         <v>33</v>
       </c>
-      <c r="K76" s="22" t="n">
-        <f aca="false">K74+1</f>
-        <v>33</v>
-      </c>
+      <c r="K76" s="22"/>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2"/>
-      <c r="B77" s="30"/>
+      <c r="B77" s="29"/>
       <c r="C77" s="22"/>
       <c r="D77" s="24"/>
       <c r="E77" s="25"/>
@@ -2403,41 +2314,38 @@
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2"/>
-      <c r="B78" s="30"/>
-      <c r="C78" s="31" t="n">
+      <c r="B78" s="29"/>
+      <c r="C78" s="30" t="n">
         <f aca="false">C76+1</f>
         <v>34</v>
       </c>
-      <c r="D78" s="32" t="n">
+      <c r="D78" s="31" t="n">
         <f aca="false">IF(D77="",D76+IF(OR(WEEKDAY(D76)=2,WEEKDAY(D76)=4),2,3),"")</f>
         <v>45975</v>
       </c>
       <c r="E78" s="25"/>
-      <c r="F78" s="33"/>
+      <c r="F78" s="32"/>
       <c r="G78" s="21"/>
       <c r="J78" s="22" t="n">
         <f aca="false">J76+1</f>
         <v>34</v>
       </c>
-      <c r="K78" s="22" t="n">
-        <f aca="false">K76+1</f>
-        <v>34</v>
-      </c>
+      <c r="K78" s="22"/>
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2"/>
-      <c r="B79" s="30"/>
-      <c r="C79" s="31"/>
-      <c r="D79" s="32"/>
+      <c r="B79" s="29"/>
+      <c r="C79" s="30"/>
+      <c r="D79" s="31"/>
       <c r="E79" s="25"/>
-      <c r="F79" s="33"/>
+      <c r="F79" s="32"/>
       <c r="G79" s="21"/>
       <c r="J79" s="22"/>
       <c r="K79" s="22"/>
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2"/>
-      <c r="B80" s="30" t="n">
+      <c r="B80" s="29" t="n">
         <v>13</v>
       </c>
       <c r="C80" s="17" t="n">
@@ -2455,14 +2363,11 @@
         <f aca="false">J78+1</f>
         <v>35</v>
       </c>
-      <c r="K80" s="22" t="n">
-        <f aca="false">K78+1</f>
-        <v>35</v>
-      </c>
+      <c r="K80" s="22"/>
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2"/>
-      <c r="B81" s="30"/>
+      <c r="B81" s="29"/>
       <c r="C81" s="17"/>
       <c r="D81" s="18"/>
       <c r="E81" s="19"/>
@@ -2473,7 +2378,7 @@
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2"/>
-      <c r="B82" s="30"/>
+      <c r="B82" s="29"/>
       <c r="C82" s="22" t="n">
         <f aca="false">C80+1</f>
         <v>36</v>
@@ -2483,64 +2388,58 @@
         <v>45980</v>
       </c>
       <c r="E82" s="25"/>
-      <c r="F82" s="35"/>
+      <c r="F82" s="34"/>
       <c r="G82" s="21"/>
       <c r="J82" s="22" t="n">
         <f aca="false">J80+1</f>
         <v>36</v>
       </c>
-      <c r="K82" s="22" t="n">
-        <f aca="false">K80+1</f>
-        <v>36</v>
-      </c>
+      <c r="K82" s="22"/>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2"/>
-      <c r="B83" s="30"/>
+      <c r="B83" s="29"/>
       <c r="C83" s="22"/>
       <c r="D83" s="24"/>
       <c r="E83" s="25"/>
-      <c r="F83" s="35"/>
+      <c r="F83" s="34"/>
       <c r="G83" s="21"/>
       <c r="J83" s="22"/>
       <c r="K83" s="22"/>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2"/>
-      <c r="B84" s="30"/>
-      <c r="C84" s="31" t="n">
+      <c r="B84" s="29"/>
+      <c r="C84" s="30" t="n">
         <f aca="false">C82+1</f>
         <v>37</v>
       </c>
-      <c r="D84" s="32" t="n">
+      <c r="D84" s="31" t="n">
         <f aca="false">IF(D83="",D82+IF(OR(WEEKDAY(D82)=2,WEEKDAY(D82)=4),2,3),"")</f>
         <v>45982</v>
       </c>
       <c r="E84" s="25"/>
-      <c r="F84" s="36"/>
+      <c r="F84" s="35"/>
       <c r="G84" s="21"/>
       <c r="J84" s="22" t="n">
         <f aca="false">J82+1</f>
         <v>37</v>
       </c>
-      <c r="K84" s="22" t="n">
-        <f aca="false">K82+1</f>
-        <v>37</v>
-      </c>
+      <c r="K84" s="22"/>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2"/>
-      <c r="B85" s="30"/>
-      <c r="C85" s="31"/>
-      <c r="D85" s="32"/>
+      <c r="B85" s="29"/>
+      <c r="C85" s="30"/>
+      <c r="D85" s="31"/>
       <c r="E85" s="25"/>
-      <c r="F85" s="36"/>
+      <c r="F85" s="35"/>
       <c r="G85" s="21"/>
       <c r="J85" s="22"/>
       <c r="K85" s="22"/>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B86" s="30" t="n">
+      <c r="B86" s="29" t="n">
         <v>14</v>
       </c>
       <c r="C86" s="17" t="n">
@@ -2558,14 +2457,11 @@
         <f aca="false">J84+1</f>
         <v>38</v>
       </c>
-      <c r="K86" s="22" t="n">
-        <f aca="false">K84+1</f>
-        <v>38</v>
-      </c>
+      <c r="K86" s="22"/>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2"/>
-      <c r="B87" s="30"/>
+      <c r="B87" s="29"/>
       <c r="C87" s="17"/>
       <c r="D87" s="18"/>
       <c r="E87" s="19"/>
@@ -2576,14 +2472,14 @@
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="2"/>
-      <c r="B88" s="30"/>
+      <c r="B88" s="29"/>
       <c r="C88" s="22"/>
       <c r="D88" s="24" t="n">
         <f aca="false">IF(D87="",D86+IF(OR(WEEKDAY(D86)=2,WEEKDAY(D86)=4),2,3),"")</f>
         <v>45987</v>
       </c>
       <c r="E88" s="25"/>
-      <c r="F88" s="37" t="s">
+      <c r="F88" s="36" t="s">
         <v>22</v>
       </c>
       <c r="G88" s="21"/>
@@ -2592,25 +2488,25 @@
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2"/>
-      <c r="B89" s="30"/>
+      <c r="B89" s="29"/>
       <c r="C89" s="22"/>
       <c r="D89" s="24"/>
       <c r="E89" s="25"/>
-      <c r="F89" s="37"/>
+      <c r="F89" s="36"/>
       <c r="G89" s="21"/>
       <c r="J89" s="22"/>
       <c r="K89" s="22"/>
     </row>
     <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="2"/>
-      <c r="B90" s="30"/>
-      <c r="C90" s="31"/>
-      <c r="D90" s="32" t="n">
+      <c r="B90" s="29"/>
+      <c r="C90" s="30"/>
+      <c r="D90" s="31" t="n">
         <f aca="false">IF(D89="",D88+IF(OR(WEEKDAY(D88)=2,WEEKDAY(D88)=4),2,3),"")</f>
         <v>45989</v>
       </c>
       <c r="E90" s="25"/>
-      <c r="F90" s="38" t="s">
+      <c r="F90" s="37" t="s">
         <v>22</v>
       </c>
       <c r="G90" s="21"/>
@@ -2619,11 +2515,11 @@
     </row>
     <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2"/>
-      <c r="B91" s="30"/>
-      <c r="C91" s="31"/>
-      <c r="D91" s="32"/>
+      <c r="B91" s="29"/>
+      <c r="C91" s="30"/>
+      <c r="D91" s="31"/>
       <c r="E91" s="25"/>
-      <c r="F91" s="38"/>
+      <c r="F91" s="37"/>
       <c r="G91" s="21"/>
       <c r="J91" s="22"/>
       <c r="K91" s="22"/>
@@ -2648,10 +2544,7 @@
         <f aca="false">J86+1</f>
         <v>39</v>
       </c>
-      <c r="K92" s="22" t="n">
-        <f aca="false">K86+1</f>
-        <v>39</v>
-      </c>
+      <c r="K92" s="22"/>
     </row>
     <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2"/>
@@ -2682,10 +2575,7 @@
         <f aca="false">J92+1</f>
         <v>40</v>
       </c>
-      <c r="K94" s="22" t="n">
-        <f aca="false">K92+1</f>
-        <v>40</v>
-      </c>
+      <c r="K94" s="22"/>
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2"/>

</xml_diff>